<commit_message>
Align IJIR v0.3.5 with complete Zenodo archive DOI
</commit_message>
<xml_diff>
--- a/06_manuscript/ijir_v0_3_5_20260728/05_tables/IJIR_Table_1_Data_Sources_v0_3_5.xlsx
+++ b/06_manuscript/ijir_v0_3_5_20260728/05_tables/IJIR_Table_1_Data_Sources_v0_3_5.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table" sheetId="1" r:id="R42c5770b9097408c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Rf1349178c2534e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table" sheetId="1" r:id="R5a0d776d4e5648b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Rf21b5b1d26c9451d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b07e991b73f4f7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15b2ceb16f4b4ca0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -549,7 +549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86bcfe0db24348ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7356dad5cba40ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize immutable v0.3.5 archive scope and DOI
</commit_message>
<xml_diff>
--- a/06_manuscript/ijir_v0_3_5_20260728/05_tables/IJIR_Table_1_Data_Sources_v0_3_5.xlsx
+++ b/06_manuscript/ijir_v0_3_5_20260728/05_tables/IJIR_Table_1_Data_Sources_v0_3_5.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table" sheetId="1" r:id="R5a0d776d4e5648b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Rf21b5b1d26c9451d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table" sheetId="1" r:id="R57a9b326b69a4ed5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="R346327e7228a454c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -509,7 +509,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15b2ceb16f4b4ca0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7b83257798e420a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -549,7 +549,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7356dad5cba40ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9beedbfa72bc4061"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>